<commit_message>
ETL: acredita autores David Fonseca y Cesar Cardozo
</commit_message>
<xml_diff>
--- a/Entrega_ETL_TecnoHogar/TecnoHogar_ETL_Taller.xlsx
+++ b/Entrega_ETL_TecnoHogar/TecnoHogar_ETL_Taller.xlsx
@@ -822,7 +822,7 @@
     <t>id_venta duplicado</t>
   </si>
   <si>
-    <t>DOCUMENTACIÓN TÉCNICA ETL — TecnoHogar Colombia S.A.S. | Arquitectura de Datos — María Celeny Pérez</t>
+    <t>DOCUMENTACIÓN TÉCNICA ETL — TecnoHogar Colombia S.A.S. | Arquitectura de Datos — María Celeny Pérez | Autores: David Fonseca y Cesar Cardozo</t>
   </si>
   <si>
     <t>1. FUENTES: Clientes(13 filas sucias), Productos(10), Vendedores(6), Ventas_Agosto(12), Ventas_Septiembre(11). Total origen: 52 filas.</t>
@@ -1756,7 +1756,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1841,7 +1841,7 @@
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1895,7 +1895,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -1949,7 +1949,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2184,7 +2184,7 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2300,7 +2300,7 @@
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2614,7 +2614,7 @@
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2905,7 +2905,7 @@
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3664,7 +3664,7 @@
   </sheetData>
   <autoFilter ref="A1:T1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3903,7 +3903,7 @@
   </sheetData>
   <autoFilter ref="A1:D1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3997,7 +3997,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4412,6 +4412,6 @@
   </sheetData>
   <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>